<commit_message>
Reframe lab around OptiPrim3; add SecurityAnalysts permission set, auditor evidence scope, admin-size guard, permission-set matrix, findings doc
</commit_message>
<xml_diff>
--- a/evidence/access-review-Q4-2026.xlsx
+++ b/evidence/access-review-Q4-2026.xlsx
@@ -18,11 +18,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sign-off" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Users'!$A$3:$J$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Groups'!$A$3:$F$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'PermissionSets'!$A$3:$G$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Assignments'!$A$3:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Q4-Review'!$A$3:$L$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Users'!$A$3:$J$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Groups'!$A$3:$F$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'PermissionSets'!$A$3:$G$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Assignments'!$A$3:$F$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Q4-Review'!$A$3:$L$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Findings'!$A$3:$K$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Remediation'!$A$3:$J$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Sign-off'!$A$3:$E$9</definedName>
@@ -515,14 +515,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Quarterly User Access Review - Q4 2026 (AWS IAM Identity Center lab)</t>
+          <t>OptiPrim3 - Quarterly User Access Review - Q4 2026 (AWS IAM Identity Center)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>EXAMPLE DATA - fictional users, IDs and tickets for a portfolio lab. Not a real organization.</t>
+          <t>EXAMPLE DATA - OptiPrim3 is a fictional company; users, IDs and tickets are made up for a portfolio lab.</t>
         </is>
       </c>
     </row>
@@ -532,7 +532,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Scope: IAM Identity Center users, groups, permission sets and account assignments for lab account 111111111111 (example).</t>
+          <t>Scope: IAM Identity Center users, groups, permission sets and account assignments for the AWS account hosting OptiPrim3's load-documentation app, 111111111111 (example: OptiPrim3 load-docs app).</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -634,7 +634,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>EXAMPLE DATA - fictional users, IDs and tickets for a portfolio lab. Not a real organization.</t>
+          <t>EXAMPLE DATA - OptiPrim3 is a fictional company; users, IDs and tickets are made up for a portfolio lab.</t>
         </is>
       </c>
     </row>
@@ -837,22 +837,22 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>mlee.auditor</t>
+          <t>jgarcia.secanalyst</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Morgan Lee</t>
+          <t>Jordan Garcia</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>IT Auditor</t>
+          <t>Security Analyst</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>ReadOnlyAuditors</t>
+          <t>SecurityAnalysts</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -861,10 +861,10 @@
         </is>
       </c>
       <c r="F7" s="6" t="n">
-        <v>46118</v>
+        <v>46216</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>46308</v>
+        <v>46310</v>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
@@ -878,29 +878,29 @@
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>REQ-09902 (joiner)</t>
+          <t>REQ-10230 (joiner)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>rpatel.dev</t>
+          <t>mlee.auditor</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Ravi Patel</t>
+          <t>Morgan Lee</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Software Developer</t>
+          <t>IT Compliance Auditor</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Developers</t>
+          <t>ReadOnlyAuditors</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -909,10 +909,10 @@
         </is>
       </c>
       <c r="F8" s="6" t="n">
-        <v>46146</v>
+        <v>46118</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>46296</v>
+        <v>46308</v>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
@@ -921,34 +921,34 @@
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>Chris Jordan</t>
+          <t>Dana Okafor</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>REQ-10011 (joiner)</t>
+          <t>REQ-09902 (joiner)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>kbrown.dev</t>
+          <t>rpatel.dev</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Kim Brown</t>
+          <t>Ravi Patel</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Software Developer</t>
+          <t>Software Developer, Load Docs</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Developers; CloudAdmins*</t>
+          <t>Developers</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -960,26 +960,74 @@
         <v>46146</v>
       </c>
       <c r="G9" s="6" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>Yes (authenticator app)</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>Chris Jordan</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>REQ-10011 (joiner)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>kbrown.dev</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Kim Brown</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Software Developer, Load Docs</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Developers; CloudAdmins*</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Enabled</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>46146</v>
+      </c>
+      <c r="G10" s="6" t="n">
         <v>46310</v>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>Yes (authenticator app)</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="I10" s="5" t="inlineStr">
         <is>
           <t>Chris Jordan</t>
         </is>
       </c>
-      <c r="J9" s="5" t="inlineStr">
+      <c r="J10" s="5" t="inlineStr">
         <is>
           <t>REQ-10012 (joiner); *CloudAdmins added in console 2026-08-21, no ticket</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:J9"/>
+  <autoFilter ref="A3:J10"/>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
@@ -993,7 +1041,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1007,7 +1055,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>EXAMPLE DATA - fictional users, IDs and tickets for a portfolio lab. Not a real organization.</t>
+          <t>EXAMPLE DATA - OptiPrim3 is a fictional company; users, IDs and tickets are made up for a portfolio lab.</t>
         </is>
       </c>
     </row>
@@ -1061,7 +1109,7 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>111111111111 (example)</t>
+          <t>111111111111 (example: OptiPrim3 load-docs app)</t>
         </is>
       </c>
       <c r="E4" s="5" t="n">
@@ -1081,7 +1129,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Cloud administrators</t>
+          <t>Cloud administrators (max 2, MFA, 1h)</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -1091,7 +1139,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>111111111111 (example)</t>
+          <t>111111111111 (example: OptiPrim3 load-docs app)</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -1108,22 +1156,22 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>ReadOnlyAuditors</t>
+          <t>SecurityAnalysts</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Internal audit / GRC</t>
+          <t>Security operations; read-only logs and findings</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>ViewOnlyAccess</t>
+          <t>SecurityAnalyst (custom)</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>111111111111 (example)</t>
+          <t>111111111111 (example: OptiPrim3 load-docs app)</t>
         </is>
       </c>
       <c r="E6" s="5" t="n">
@@ -1138,35 +1186,65 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
+          <t>ReadOnlyAuditors</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Internal audit / GRC; approved evidence only</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>ViewOnlyAccess (+ evidence prefix read)</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>111111111111 (example: OptiPrim3 load-docs app)</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Compliance Manager (Sam Ortiz)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
           <t>Developers</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Application developers</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>ReadOnlyAccess</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>111111111111 (example)</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="n">
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>111111111111 (example: OptiPrim3 load-docs app)</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>Chris Jordan</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:F7"/>
+  <autoFilter ref="A3:F8"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
@@ -1180,7 +1258,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1195,7 +1273,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>EXAMPLE DATA - fictional users, IDs and tickets for a portfolio lab. Not a real organization.</t>
+          <t>EXAMPLE DATA - OptiPrim3 is a fictional company; users, IDs and tickets are made up for a portfolio lab.</t>
         </is>
       </c>
     </row>
@@ -1313,17 +1391,17 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>ReadOnlyAccess</t>
+          <t>SecurityAnalyst</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>AWS managed</t>
+          <t>Custom inline</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>ReadOnlyAccess</t>
+          <t>Read CloudTrail (LookupEvents, trails), CloudWatch Logs (read + Insights queries), GuardDuty/Security Hub/Config/Access Analyzer Get/List/Describe; explicit Deny on stopping/deleting/updating any of them and all IAM/SSO</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -1333,7 +1411,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Developers</t>
+          <t>SecurityAnalysts</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
@@ -1343,49 +1421,86 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Can read data (e.g. S3 objects)</t>
+          <t>Sees sensitive security data; cannot alter it</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
+          <t>ReadOnlyAccess</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>AWS managed</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>ReadOnlyAccess</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>4 hours</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Developers</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Can read data (e.g. S3 load documents)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
           <t>ViewOnlyAccess</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>AWS managed</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>job-function/ViewOnlyAccess</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>AWS managed + optional inline</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>job-function/ViewOnlyAccess; optional inline read on s3://&lt;evidence bucket&gt;/approved-evidence/* with Deny on writes</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>2 hours</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>ReadOnlyAuditors</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>Metadata only; suits audit</t>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Metadata plus approved evidence only</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:G7"/>
+  <autoFilter ref="A3:G8"/>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
@@ -1399,7 +1514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1413,7 +1528,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>EXAMPLE DATA - fictional users, IDs and tickets for a portfolio lab. Not a real organization.</t>
+          <t>EXAMPLE DATA - OptiPrim3 is a fictional company; users, IDs and tickets are made up for a portfolio lab.</t>
         </is>
       </c>
     </row>
@@ -1467,7 +1582,7 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>111111111111 (example)</t>
+          <t>111111111111 (example: OptiPrim3 load-docs app)</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -1499,7 +1614,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>111111111111 (example)</t>
+          <t>111111111111 (example: OptiPrim3 load-docs app)</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -1531,7 +1646,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>111111111111 (example)</t>
+          <t>111111111111 (example: OptiPrim3 load-docs app)</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -1548,22 +1663,22 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>mlee.auditor</t>
+          <t>jgarcia.secanalyst</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>ReadOnlyAuditors</t>
+          <t>SecurityAnalysts</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>ViewOnlyAccess</t>
+          <t>SecurityAnalyst</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>111111111111 (example)</t>
+          <t>111111111111 (example: OptiPrim3 load-docs app)</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -1580,22 +1695,22 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>rpatel.dev</t>
+          <t>mlee.auditor</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Developers</t>
+          <t>ReadOnlyAuditors</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>ReadOnlyAccess</t>
+          <t>ViewOnlyAccess</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>111111111111 (example)</t>
+          <t>111111111111 (example: OptiPrim3 load-docs app)</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -1612,7 +1727,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>kbrown.dev</t>
+          <t>rpatel.dev</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -1627,7 +1742,7 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>111111111111 (example)</t>
+          <t>111111111111 (example: OptiPrim3 load-docs app)</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -1649,32 +1764,64 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
+          <t>Developers</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>ReadOnlyAccess</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>111111111111 (example: OptiPrim3 load-docs app)</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Via group</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>kbrown.dev</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
           <t>CloudAdmins</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>AdministratorAccess</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>111111111111 (example)</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>111111111111 (example: OptiPrim3 load-docs app)</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>Via group</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t>No - console drift</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:F10"/>
+  <autoFilter ref="A3:F11"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
@@ -1688,7 +1835,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1708,7 +1855,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>EXAMPLE DATA - fictional users, IDs and tickets for a portfolio lab. Not a real organization.</t>
+          <t>EXAMPLE DATA - OptiPrim3 is a fictional company; users, IDs and tickets are made up for a portfolio lab.</t>
         </is>
       </c>
     </row>
@@ -1989,7 +2136,7 @@
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>Audit role; view-only appropriate</t>
+          <t>Audit role; view-only plus approved evidence appropriate</t>
         </is>
       </c>
       <c r="J7" s="6" t="n">
@@ -2014,21 +2161,21 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>rpatel.dev</t>
+          <t>jgarcia.secanalyst</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Developers</t>
+          <t>SecurityAnalysts</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>ReadOnlyAccess</t>
+          <t>SecurityAnalyst</t>
         </is>
       </c>
       <c r="E8" s="6" t="n">
-        <v>46296</v>
+        <v>46310</v>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
@@ -2037,7 +2184,7 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Chris Jordan</t>
+          <t>Dana Okafor</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
@@ -2047,15 +2194,15 @@
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>Active developer</t>
+          <t>SOC analyst; read-only to logs and findings matches role</t>
         </is>
       </c>
       <c r="J8" s="6" t="n">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="K8" s="5" t="inlineStr">
         <is>
-          <t>REQ-10564</t>
+          <t>REQ-10568</t>
         </is>
       </c>
       <c r="L8" s="5" t="inlineStr">
@@ -2072,7 +2219,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>kbrown.dev</t>
+          <t>rpatel.dev</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -2086,7 +2233,7 @@
         </is>
       </c>
       <c r="E9" s="6" t="n">
-        <v>46310</v>
+        <v>46296</v>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
@@ -2113,7 +2260,7 @@
       </c>
       <c r="K9" s="5" t="inlineStr">
         <is>
-          <t>REQ-10565</t>
+          <t>REQ-10564</t>
         </is>
       </c>
       <c r="L9" s="5" t="inlineStr">
@@ -2135,12 +2282,12 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>CloudAdmins</t>
+          <t>Developers</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>AdministratorAccess</t>
+          <t>ReadOnlyAccess</t>
         </is>
       </c>
       <c r="E10" s="6" t="n">
@@ -2153,17 +2300,17 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Dana Okafor</t>
+          <t>Chris Jordan</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Revoke</t>
+          <t>Keep</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>Added in console during an outage with no ticket or approval; developer role does not need admin</t>
+          <t>Active developer</t>
         </is>
       </c>
       <c r="J10" s="6" t="n">
@@ -2171,17 +2318,75 @@
       </c>
       <c r="K10" s="5" t="inlineStr">
         <is>
+          <t>REQ-10565</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>AR-Q4-008</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>kbrown.dev</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>CloudAdmins</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>AdministratorAccess</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>46310</v>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Yes (authenticator app)</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Dana Okafor</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Revoke</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>Added in console during an outage with no ticket or approval; developer role does not need admin</t>
+        </is>
+      </c>
+      <c r="J11" s="6" t="n">
+        <v>46309</v>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
           <t>REQ-10566</t>
         </is>
       </c>
-      <c r="L10" s="5" t="inlineStr">
+      <c r="L11" s="5" t="inlineStr">
         <is>
           <t>Remediating</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:L10"/>
+  <autoFilter ref="A3:L11"/>
   <mergeCells count="1">
     <mergeCell ref="A1:L1"/>
   </mergeCells>
@@ -2230,7 +2435,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>EXAMPLE DATA - fictional users, IDs and tickets for a portfolio lab. Not a real organization.</t>
+          <t>EXAMPLE DATA - OptiPrim3 is a fictional company; users, IDs and tickets are made up for a portfolio lab.</t>
         </is>
       </c>
     </row>
@@ -2439,7 +2644,7 @@
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>Save a CloudTrail Lake / Athena or CLI query in the build checklist for the next review</t>
+          <t>Save a CloudTrail CLI query (lookup-events) in the build checklist; have SecurityAnalysts run it each quarter</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
@@ -2494,7 +2699,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>EXAMPLE DATA - fictional users, IDs and tickets for a portfolio lab. Not a real organization.</t>
+          <t>EXAMPLE DATA - OptiPrim3 is a fictional company; users, IDs and tickets are made up for a portfolio lab.</t>
         </is>
       </c>
     </row>
@@ -2787,7 +2992,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>EXAMPLE DATA - fictional users, IDs and tickets for a portfolio lab. Not a real organization.</t>
+          <t>EXAMPLE DATA - OptiPrim3 is a fictional company; users, IDs and tickets are made up for a portfolio lab.</t>
         </is>
       </c>
     </row>
@@ -2871,7 +3076,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Reviewer - CloudAdmins / Auditors</t>
+          <t>Reviewer - CloudAdmins / SecurityAnalysts / Auditors</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -2881,7 +3086,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>I reviewed all privileged and audit entitlements and recorded a decision for each.</t>
+          <t>I reviewed all privileged, security and audit entitlements and recorded a decision for each.</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">

</xml_diff>